<commit_message>
Fixed some column definitions
</commit_message>
<xml_diff>
--- a/Data/final_tables/supplementary_file_3_BARD1_all_reagents.xlsx
+++ b/Data/final_tables/supplementary_file_3_BARD1_all_reagents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivan/Documents/GitHub/BARD1_SGE_analysis/Data/final_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB6212C-F38E-224B-827F-E7DCA9DEFE31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D6AB3A1-33A0-1043-98AA-3B8540DF01FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16100" xr2:uid="{D2A65EDD-B858-E447-8FDB-B7AA24207239}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16100" activeTab="6" xr2:uid="{D2A65EDD-B858-E447-8FDB-B7AA24207239}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="7" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="1273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="1271">
   <si>
     <t>Oligo Name</t>
   </si>
@@ -3093,9 +3093,6 @@
   </si>
   <si>
     <t>CCCACAAATAGAAGTAGCATCCATCA</t>
-  </si>
-  <si>
-    <t>Full Seqeunce</t>
   </si>
   <si>
     <t>BARD1_X1_RNA_PCR2_Fwd</t>
@@ -5665,9 +5662,6 @@
   </si>
   <si>
     <t>Denotes if primer is a forward (FWD) or reverse (REV) primer</t>
-  </si>
-  <si>
-    <t>sequence Name</t>
   </si>
   <si>
     <t>Name of oligo. Typically they are: SGE region following by the Illumina adapter added</t>
@@ -6206,79 +6200,79 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B2" t="s">
         <v>1227</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1228</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
+        <v>1228</v>
+      </c>
+      <c r="B3" t="s">
         <v>1229</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1230</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
+        <v>1230</v>
+      </c>
+      <c r="B5" t="s">
         <v>1231</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1232</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B6" t="s">
         <v>1233</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1234</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B7" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B8" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B11" t="s">
         <v>1238</v>
-      </c>
-      <c r="B11" t="s">
-        <v>1239</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B12" t="s">
         <v>1233</v>
-      </c>
-      <c r="B12" t="s">
-        <v>1234</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="182" customHeight="1" x14ac:dyDescent="0.2">
@@ -6286,7 +6280,7 @@
         <v>37</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -6294,37 +6288,37 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -6332,23 +6326,23 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B23" t="s">
         <v>1249</v>
-      </c>
-      <c r="B23" t="s">
-        <v>1250</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B24" t="s">
         <v>1233</v>
-      </c>
-      <c r="B24" t="s">
-        <v>1234</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="153" x14ac:dyDescent="0.2">
@@ -6356,7 +6350,7 @@
         <v>764</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -6364,23 +6358,23 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B28" t="s">
         <v>1252</v>
-      </c>
-      <c r="B28" t="s">
-        <v>1253</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B29" t="s">
         <v>1233</v>
-      </c>
-      <c r="B29" t="s">
-        <v>1234</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="188" x14ac:dyDescent="0.2">
@@ -6388,7 +6382,7 @@
         <v>813</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -6396,55 +6390,55 @@
         <v>814</v>
       </c>
       <c r="B31" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>1255</v>
+        <v>764</v>
       </c>
       <c r="B32" t="s">
-        <v>1256</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
         <v>1255</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1257</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="B35" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="B36" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B37" t="s">
-        <v>1261</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B38" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -6452,23 +6446,23 @@
         <v>1</v>
       </c>
       <c r="B39" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="B41" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B42" t="s">
         <v>1233</v>
-      </c>
-      <c r="B42" t="s">
-        <v>1234</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
@@ -6476,7 +6470,7 @@
         <v>37</v>
       </c>
       <c r="B43" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -6484,35 +6478,35 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>1266</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="B49" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
     </row>
   </sheetData>
@@ -6533,54 +6527,54 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>1111</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>1112</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1113</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>1114</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1187</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>1115</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>1116</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>1117</v>
-      </c>
       <c r="C3" s="4" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>1119</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>1120</v>
       </c>
       <c r="C5" s="4">
         <v>636767</v>
@@ -6588,68 +6582,68 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>1122</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>1123</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>1124</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>1125</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>1126</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>1127</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>1128</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>1129</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>1130</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>1131</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>1129</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>1132</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>1133</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>1134</v>
       </c>
       <c r="C11" s="4">
         <v>80204</v>
@@ -6657,10 +6651,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="C12" s="4">
         <v>69506</v>
@@ -6668,10 +6662,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>1136</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>1137</v>
       </c>
       <c r="C13" s="4">
         <v>7958935001</v>
@@ -6679,10 +6673,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>1138</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>1139</v>
       </c>
       <c r="C14" s="4">
         <v>29343057</v>
@@ -6690,43 +6684,43 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>1140</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>1141</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>1142</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>1143</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>1144</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>1145</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>1146</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>1147</v>
       </c>
       <c r="C18" s="4">
         <v>18090200</v>
@@ -6734,10 +6728,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>1148</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>1149</v>
       </c>
       <c r="C19" s="4">
         <v>12440079</v>
@@ -6745,21 +6739,21 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>1150</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>1151</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>1152</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="C21" s="4">
         <v>10010072</v>
@@ -6767,10 +6761,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="C22" s="4">
         <v>25200114</v>
@@ -6778,32 +6772,32 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>1155</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>1149</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>1156</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>1157</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>1149</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>1158</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="C25" s="4">
         <v>631318</v>
@@ -6811,109 +6805,109 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>1160</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="C26" s="4" t="s">
         <v>1161</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>1162</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>1163</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>1161</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>1164</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>1165</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>1147</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>1166</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>1167</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>1147</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>1168</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C30" s="4" t="s">
         <v>1169</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>1170</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>1171</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>1172</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>1173</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>1174</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>1175</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>1176</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>1177</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="C35" s="4">
         <v>10777019</v>
@@ -6921,35 +6915,35 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>1180</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>1181</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>1182</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>1183</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>1184</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>1147</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>1185</v>
       </c>
     </row>
   </sheetData>
@@ -6985,7 +6979,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -7092,7 +7086,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -7199,7 +7193,7 @@
         <v>36</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -7306,7 +7300,7 @@
         <v>4</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -7413,7 +7407,7 @@
         <v>5</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -7507,7 +7501,7 @@
         <v>6</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -7547,7 +7541,7 @@
         <v>6</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -7606,7 +7600,7 @@
         <v>7</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -7713,7 +7707,7 @@
         <v>8</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -7820,7 +7814,7 @@
         <v>9</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -7927,7 +7921,7 @@
         <v>10</v>
       </c>
       <c r="C125" s="6" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -8034,7 +8028,7 @@
         <v>11</v>
       </c>
       <c r="C139" s="6" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -8141,7 +8135,7 @@
         <v>12</v>
       </c>
       <c r="C153" s="6" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -8248,7 +8242,7 @@
         <v>13</v>
       </c>
       <c r="C167" s="6" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
@@ -8355,7 +8349,7 @@
         <v>14</v>
       </c>
       <c r="C181" s="6" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.2">
@@ -8462,7 +8456,7 @@
         <v>15</v>
       </c>
       <c r="C195" s="6" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.2">
@@ -8569,7 +8563,7 @@
         <v>16</v>
       </c>
       <c r="C209" s="6" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.2">
@@ -8676,7 +8670,7 @@
         <v>17</v>
       </c>
       <c r="C223" s="6" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.2">
@@ -8783,7 +8777,7 @@
         <v>18</v>
       </c>
       <c r="C237" s="6" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.2">
@@ -8874,7 +8868,7 @@
         <v>19</v>
       </c>
       <c r="C249" s="6" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.2">
@@ -8965,7 +8959,7 @@
         <v>20</v>
       </c>
       <c r="C261" s="6" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.2">
@@ -9072,7 +9066,7 @@
         <v>21</v>
       </c>
       <c r="C275" s="6" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.2">
@@ -9179,7 +9173,7 @@
         <v>22</v>
       </c>
       <c r="C289" s="6" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.2">
@@ -9286,7 +9280,7 @@
         <v>23</v>
       </c>
       <c r="C303" s="6" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.2">
@@ -9377,7 +9371,7 @@
         <v>24</v>
       </c>
       <c r="C315" s="6" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.2">
@@ -9468,7 +9462,7 @@
         <v>25</v>
       </c>
       <c r="C327" s="6" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.2">
@@ -9559,7 +9553,7 @@
         <v>26</v>
       </c>
       <c r="C339" s="6" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.2">
@@ -9650,7 +9644,7 @@
         <v>27</v>
       </c>
       <c r="C351" s="6" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.2">
@@ -9741,7 +9735,7 @@
         <v>28</v>
       </c>
       <c r="C363" s="6" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.2">
@@ -9832,7 +9826,7 @@
         <v>29</v>
       </c>
       <c r="C375" s="6" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="376" spans="1:3" x14ac:dyDescent="0.2">
@@ -9923,7 +9917,7 @@
         <v>30</v>
       </c>
       <c r="C387" s="6" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.2">
@@ -10105,7 +10099,7 @@
         <v>33</v>
       </c>
       <c r="C411" s="6" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="412" spans="1:3" x14ac:dyDescent="0.2">
@@ -10212,7 +10206,7 @@
         <v>34</v>
       </c>
       <c r="C425" s="6" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.2">
@@ -10319,7 +10313,7 @@
         <v>35</v>
       </c>
       <c r="C439" s="6" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="440" spans="1:3" x14ac:dyDescent="0.2">
@@ -11720,10 +11714,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -11731,43 +11725,43 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>1014</v>
@@ -11775,10 +11769,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>1015</v>
@@ -11786,10 +11780,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>1016</v>
@@ -11818,18 +11812,18 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1017</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>1223</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>1224</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>1225</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -11837,10 +11831,10 @@
         <v>1005</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>1018</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -11848,10 +11842,10 @@
         <v>1005</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>1020</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>1021</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -11859,10 +11853,10 @@
         <v>1006</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>1022</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>1023</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -11870,10 +11864,10 @@
         <v>1006</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>1024</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>1025</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -11881,10 +11875,10 @@
         <v>1007</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>1026</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>1027</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -11892,194 +11886,194 @@
         <v>1007</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>1028</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>1029</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>1030</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>1031</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>1032</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>1033</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>1034</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>1035</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>1036</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>1037</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>1038</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>1039</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>1040</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>1041</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>1042</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>1043</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>1044</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>1045</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>1046</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>1047</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>1048</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>1049</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>1050</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>1051</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>1052</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>1053</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>1054</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>1055</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>1056</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>1057</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>1058</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -12087,10 +12081,10 @@
         <v>1008</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>1059</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>1060</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -12098,10 +12092,10 @@
         <v>1008</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>1060</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>1061</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>1062</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -12109,10 +12103,10 @@
         <v>1009</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>1063</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -12120,10 +12114,10 @@
         <v>1009</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>1065</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>1066</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -12131,10 +12125,10 @@
         <v>1010</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>1067</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>1068</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -12142,10 +12136,10 @@
         <v>1010</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>1069</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>1070</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -12153,10 +12147,10 @@
         <v>1011</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>1071</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>1072</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -12164,10 +12158,10 @@
         <v>1011</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>1073</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>1074</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -12175,10 +12169,10 @@
         <v>1012</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>1075</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>1076</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -12186,10 +12180,10 @@
         <v>1012</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>1077</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>1078</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -12197,10 +12191,10 @@
         <v>1013</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>1079</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>1080</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -12208,29 +12202,29 @@
         <v>1013</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>1081</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>1082</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>1083</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>1084</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>1085</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>751</v>
@@ -12238,56 +12232,56 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B56" s="2" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>1087</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>1088</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>1089</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>1090</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>1091</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>1092</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>1093</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>1094</v>
       </c>
     </row>
   </sheetData>

</xml_diff>